<commit_message>
EPBDS-16835 Fix DateRange reading only US dates and splitting an ISO date at its dashes, which failed ISO ranges
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ValuesAndRanges.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ValuesAndRanges.xlsx
@@ -20,10 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -164,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,13 +186,16 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -772,7 +774,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D18" s="13" t="n">
         <v>45306.4375</v>
       </c>
       <c r="E18" s="5" t="n"/>
@@ -1092,7 +1094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:J50"/>
+  <dimension ref="B2:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1553,10 +1555,10 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1">
+    <row r="38" ht="30" customHeight="1">
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>The same forms work for the other range types. A DoubleRange accepts fractions; a StringRange compares the numbers inside texts as numbers; a DateRange accepts dates with an optional time.</t>
+          <t>The same forms work for the other range types. A DoubleRange accepts fractions; a StringRange compares the numbers inside texts as numbers; a DateRange accepts ISO dates "2024-12-31" and US dates "12/31/2024" with an optional time, written after a space or, in the ISO form, after a "T".</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1806,7 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>01/01/2024 - 12/31/2024</t>
+          <t>2024-01-01 - 2024-12-31</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
@@ -1849,7 +1851,7 @@
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>[01/01/2024; 06/30/2024)</t>
+          <t>[2024-01-01; 2024-06-30)</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
@@ -1903,6 +1905,51 @@
         </is>
       </c>
       <c r="J50" s="12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>[0.5; 1.5)</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>a - f</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>A1 - A10</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>&lt;= 2024-05-31T23:59:59</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-01</t>
+        </is>
+      </c>
+      <c r="J51" s="12" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -3778,7 +3825,7 @@
     <row r="107" ht="43.5" customHeight="1">
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>A DateRange accepts dates in the US form "12/31/2024" with an optional time "12/31/2024 23:59:59". A single date can also be an Excel date cell. A single date matches only that moment. "+", "and more", "or less", "&lt;", "&lt;=" and the other forms work as for numbers. A border without a time is the start of the day.</t>
+          <t>A DateRange accepts dates in the ISO form "2024-12-31" or in the US form "12/31/2024", with an optional time "2024-12-31 23:59:59". A single date can also be an Excel date cell, and it matches only that moment. "+", "and more", "or less", "&lt;", "&lt;=" and the other forms work as for numbers. A border without a time is the start of the day.</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3862,7 @@
     <row r="112">
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="C112" s="12" t="inlineStr">
@@ -3827,7 +3874,7 @@
     <row r="113">
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>02/01/2024 - 02/29/2024</t>
+          <t>2024-02-01 - 2024-02-29</t>
         </is>
       </c>
       <c r="C113" s="12" t="inlineStr">
@@ -3851,7 +3898,7 @@
     <row r="115">
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>04/01/2024 ... 04/30/2024</t>
+          <t>2024-04-01 ... 2024-04-30</t>
         </is>
       </c>
       <c r="C115" s="12" t="inlineStr">
@@ -3863,7 +3910,7 @@
     <row r="116">
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>[05/01/2024; 06/01/2024)</t>
+          <t>[2024-05-01; 2024-06-01)</t>
         </is>
       </c>
       <c r="C116" s="12" t="inlineStr">
@@ -3875,7 +3922,7 @@
     <row r="117">
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>(06/01/2024 .. 06/30/2024 23:59:59]</t>
+          <t>(2024-06-01 .. 2024-06-30 23:59:59]</t>
         </is>
       </c>
       <c r="C117" s="12" t="inlineStr">
@@ -3899,7 +3946,7 @@
     <row r="119">
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>&lt; 09/01/2024 &gt;= 08/01/2024</t>
+          <t>&lt; 2024-09-01 &gt;= 2024-08-01</t>
         </is>
       </c>
       <c r="C119" s="12" t="inlineStr">
@@ -3911,7 +3958,7 @@
     <row r="120">
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>12/01/2024 +</t>
+          <t>2024-12-01 +</t>
         </is>
       </c>
       <c r="C120" s="12" t="inlineStr">
@@ -3935,7 +3982,7 @@
     <row r="122">
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>more than 10/15/2024</t>
+          <t>more than 2024-10-15</t>
         </is>
       </c>
       <c r="C122" s="12" t="inlineStr">
@@ -3959,7 +4006,7 @@
     <row r="124">
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>06/30/2020 or less</t>
+          <t>2020-06-30 or less</t>
         </is>
       </c>
       <c r="C124" s="12" t="inlineStr">
@@ -3971,7 +4018,7 @@
     <row r="125">
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>&lt; 01/01/2023</t>
+          <t>&lt; 2023-01-01</t>
         </is>
       </c>
       <c r="C125" s="12" t="inlineStr">
@@ -4045,7 +4092,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="B133" s="10" t="n">
+      <c r="B133" s="13" t="n">
         <v>45292.41666666666</v>
       </c>
       <c r="C133" s="12" t="n"/>
@@ -4093,7 +4140,7 @@
       <c r="C138" s="12" t="n"/>
     </row>
     <row r="139">
-      <c r="B139" s="10" t="n">
+      <c r="B139" s="13" t="n">
         <v>45473.95833333334</v>
       </c>
       <c r="C139" s="12" t="inlineStr">
@@ -4221,7 +4268,7 @@
     <row r="153">
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>[01/01/2024; 04/01/2024)</t>
+          <t>[2024-01-01; 2024-04-01)</t>
         </is>
       </c>
       <c r="C153" s="12" t="inlineStr">
@@ -4233,7 +4280,7 @@
     <row r="154">
       <c r="B154" s="5" t="inlineStr">
         <is>
-          <t>&gt;= 04/01/2024 &lt; 07/01/2024</t>
+          <t>&gt;= 2024-04-01 &lt; 2024-07-01</t>
         </is>
       </c>
       <c r="C154" s="12" t="inlineStr">
@@ -4245,7 +4292,7 @@
     <row r="155">
       <c r="B155" s="5" t="inlineStr">
         <is>
-          <t>07/01/2024 - 09/30/2024 23:59:59</t>
+          <t>2024-07-01 - 2024-09-30 23:59:59</t>
         </is>
       </c>
       <c r="C155" s="12" t="inlineStr">
@@ -4257,7 +4304,7 @@
     <row r="156">
       <c r="B156" s="5" t="inlineStr">
         <is>
-          <t>10/01/2024 and more</t>
+          <t>2024-10-01 and more</t>
         </is>
       </c>
       <c r="C156" s="12" t="inlineStr">
@@ -4319,7 +4366,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="B163" s="10" t="n">
+      <c r="B163" s="13" t="n">
         <v>45565.75</v>
       </c>
       <c r="C163" s="12" t="inlineStr">
@@ -4346,11 +4393,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B109:C109"/>
     <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B69:C69"/>
     <mergeCell ref="B53:I53"/>
-    <mergeCell ref="B109:C109"/>
     <mergeCell ref="B91:I91"/>
     <mergeCell ref="B151:C151"/>
     <mergeCell ref="B19:C19"/>
@@ -4824,7 +4871,7 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>= new DateRange("&gt;= 01/01/2017 &lt; 01/01/2019").toString()</t>
+          <t>= new DateRange("&gt;= 2017-01-01 &lt; 2019-01-01").toString()</t>
         </is>
       </c>
     </row>
@@ -4981,7 +5028,7 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>new DateRange("&gt;= 01/01/2017 &lt; 01/01/2019").toString()</t>
+          <t>new DateRange("&gt;= 2017-01-01 &lt; 2019-01-01").toString()</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">

</xml_diff>

<commit_message>
EPBDS-9967 Restore $, thousands separators and K, M, B in ranges, not formulas
A comma in a range has to separate groups of three digits now, so 77,99 is a
list instead of 7799, and a K, M, B bound of a DoubleRange is exact.
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ValuesAndRanges.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ValuesAndRanges.xlsx
@@ -1094,7 +1094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:J51"/>
+  <dimension ref="B2:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1119,7 +1119,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>IntRange and DoubleRange hold intervals of numbers, CharRange of characters, StringRange of texts and DateRange of dates. A cell or "new IntRange(text)" accepts the forms below. Square brackets include a border, round brackets exclude it. "a .. b" includes both borders, "a ... b" excludes both, "a - b" includes both.</t>
+          <t>IntRange and DoubleRange hold intervals of numbers, CharRange of characters, StringRange of texts and DateRange of dates. A cell or "new IntRange(text)" accepts the forms below. Square brackets include a border, round brackets exclude it. "a .. b" includes both borders, "a ... b" excludes both, "a - b" includes both. A number border may start with "$", group its thousands with commas and end with a K, M or B multiplier: "$1,000 - $2,000" or "[1K .. 1M)". A comma must separate groups of three digits.</t>
         </is>
       </c>
     </row>
@@ -1543,291 +1543,201 @@
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
+          <t>$1,000 - $2,000</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>[1K .. 1M)</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>999999</v>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C36" s="5" t="n">
+      <c r="C39" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>The same forms work for the other range types. A DoubleRange accepts fractions; a StringRange compares the numbers inside texts as numbers; a DateRange accepts ISO dates "2024-12-31" and US dates "12/31/2024" with an optional time, written after a space or, in the ISO form, after a "T".</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Method Boolean OtherRangesHave(DoubleRange amounts, Double amount, CharRange letters, Character letter, StringRange codes, String code, DateRange period, Date day)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>return contains(amounts, amount) &amp;&amp; contains(letters, letter) &amp;&amp; contains(codes, code) &amp;&amp; contains(period, day);</t>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>The same forms work for the other range types. A DoubleRange accepts fractions, also before a multiplier: "2.5K" is 2500. A StringRange compares the numbers inside texts as numbers; a DateRange accepts ISO dates "2024-12-31" and US dates "12/31/2024" with an optional time, written after a space or, in the ISO form, after a "T".</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="3" t="inlineStr">
         <is>
+          <t>Method Boolean OtherRangesHave(DoubleRange amounts, Double amount, CharRange letters, Character letter, StringRange codes, String code, DateRange period, Date day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>return contains(amounts, amount) &amp;&amp; contains(letters, letter) &amp;&amp; contains(codes, code) &amp;&amp; contains(period, day);</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
           <t>Test OtherRangesHave OtherRangesHaveTest</t>
         </is>
       </c>
-      <c r="C43" s="6" t="n"/>
-      <c r="D43" s="6" t="n"/>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="6" t="n"/>
-      <c r="G43" s="6" t="n"/>
-      <c r="H43" s="6" t="n"/>
-      <c r="I43" s="6" t="n"/>
-      <c r="J43" s="4" t="n"/>
-    </row>
-    <row r="44">
-      <c r="B44" s="7" t="inlineStr">
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
+      <c r="I46" s="6" t="n"/>
+      <c r="J46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>amounts</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="D44" s="7" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>letters</t>
         </is>
       </c>
-      <c r="E44" s="7" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>letter</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>codes</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H47" s="7" t="inlineStr">
         <is>
           <t>period</t>
         </is>
       </c>
-      <c r="I44" s="7" t="inlineStr">
+      <c r="I47" s="7" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="J44" s="7" t="inlineStr">
+      <c r="J47" s="7" t="inlineStr">
         <is>
           <t>_res_</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="8" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>Amounts</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="C48" s="8" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>Letters</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>Letter</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
+      <c r="F48" s="8" t="inlineStr">
         <is>
           <t>Codes</t>
         </is>
       </c>
-      <c r="G45" s="8" t="inlineStr">
+      <c r="G48" s="8" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="H45" s="8" t="inlineStr">
+      <c r="H48" s="8" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="I45" s="8" t="inlineStr">
+      <c r="I48" s="8" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="J45" s="8" t="inlineStr">
+      <c r="J48" s="8" t="inlineStr">
         <is>
           <t>All Contain</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>[0.5; 1.5)</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>a - f</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>A1 - A10</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>01/01/2024 - 12/31/2024</t>
-        </is>
-      </c>
-      <c r="I46" s="5" t="inlineStr">
-        <is>
-          <t>2024-06-01</t>
-        </is>
-      </c>
-      <c r="J46" s="12" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>[0.5; 1.5)</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>a - f</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>A1 - A10</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>01/01/2024 - 12/31/2024</t>
-        </is>
-      </c>
-      <c r="I47" s="5" t="inlineStr">
-        <is>
-          <t>2024-06-01</t>
-        </is>
-      </c>
-      <c r="J47" s="12" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>&gt;= 2.5</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>[a; f)</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>f</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>A1 - A10</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>2024-01-01 - 2024-12-31</t>
-        </is>
-      </c>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>2024-06-01</t>
-        </is>
-      </c>
-      <c r="J48" s="12" t="inlineStr">
-        <is>
-          <t>false</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>&gt;= 2.5</t>
+          <t>[0.5; 1.5)</t>
         </is>
       </c>
       <c r="C49" s="5" t="n">
-        <v>3.1</v>
+        <v>0.75</v>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
@@ -1836,27 +1746,27 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>c</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>&gt;= AA &lt; DD</t>
+          <t>A1 - A10</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>B7</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>[2024-01-01; 2024-06-30)</t>
+          <t>01/01/2024 - 12/31/2024</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>2024-06-29</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="J49" s="12" t="inlineStr">
@@ -1868,11 +1778,11 @@
     <row r="50">
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>&gt;= 2.5</t>
+          <t>[0.5; 1.5)</t>
         </is>
       </c>
       <c r="C50" s="5" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
@@ -1881,7 +1791,7 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>c</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -1891,7 +1801,7 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>A22</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
@@ -1913,53 +1823,233 @@
     <row r="51">
       <c r="B51" s="5" t="inlineStr">
         <is>
+          <t>&gt;= 2.5</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>[a; f)</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>A1 - A10</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>2024-01-01 - 2024-12-31</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-01</t>
+        </is>
+      </c>
+      <c r="J51" s="12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>&gt;= 2.5</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>a - f</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>&gt;= AA &lt; DD</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>[2024-01-01; 2024-06-30)</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-29</t>
+        </is>
+      </c>
+      <c r="J52" s="12" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>&gt;= 2.5</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>a - f</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>A1 - A10</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>A22</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>01/01/2024 - 12/31/2024</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-01</t>
+        </is>
+      </c>
+      <c r="J53" s="12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="5" t="inlineStr">
+        <is>
           <t>[0.5; 1.5)</t>
         </is>
       </c>
-      <c r="C51" s="5" t="n">
+      <c r="C54" s="5" t="n">
         <v>0.75</v>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>a - f</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>A1 - A10</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="H51" s="5" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>&lt;= 2024-05-31T23:59:59</t>
         </is>
       </c>
-      <c r="I51" s="5" t="inlineStr">
+      <c r="I54" s="5" t="inlineStr">
         <is>
           <t>2024-06-01</t>
         </is>
       </c>
-      <c r="J51" s="12" t="inlineStr">
+      <c r="J54" s="12" t="inlineStr">
         <is>
           <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>[$2.5K; 1.5M)</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>a - f</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>A1 - A10</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>01/01/2024 - 12/31/2024</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-01</t>
+        </is>
+      </c>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B43:J43"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B46:J46"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1973,7 +2063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I74"/>
+  <dimension ref="B2:E93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -2705,15 +2795,185 @@
       </c>
       <c r="D74" s="12" t="n"/>
     </row>
+    <row r="76" ht="57" customHeight="1">
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Number borders can be written the way amounts are: "$1,000" is 1000 and "2.5K" is 2500, while a whole-number parameter takes whole borders only. A comma between groups of three digits groups thousands in a column of ranges, as in "&lt; $1,000" or "2,500 - 1M". A column with a list, such as "1, 3" or "77,99", reads every comma as a separator, so write big numbers there without commas. Formulas do not accept these forms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>SmartRules String AmountBand(Double amount)</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Band</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>&lt; $1,000</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>[1K .. 2.5K)</t>
+        </is>
+      </c>
+      <c r="C81" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>2,500 - 1M</t>
+        </is>
+      </c>
+      <c r="C82" s="12" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>&gt; 1M</t>
+        </is>
+      </c>
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>Huge</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Test AmountBand AmountBandTest</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Band</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="5" t="n">
+        <v>999.99</v>
+      </c>
+      <c r="C88" s="12" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="5" t="n">
+        <v>2499.99</v>
+      </c>
+      <c r="C90" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="5" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C91" s="12" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="C92" s="12" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="5" t="n">
+        <v>1000000.01</v>
+      </c>
+      <c r="C93" s="12" t="inlineStr">
+        <is>
+          <t>Huge</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="12">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B78:C78"/>
     <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B85:C85"/>
     <mergeCell ref="B36:I36"/>
     <mergeCell ref="B59:E59"/>
     <mergeCell ref="B65:D65"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B76:I76"/>
     <mergeCell ref="B57:I57"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>

</xml_diff>